<commit_message>
Modelo correcto y archivos excel actualizados
</commit_message>
<xml_diff>
--- a/RESULTADOS.xlsx
+++ b/RESULTADOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frsfutneduar-my.sharepoint.com/personal/lzeballos_frsf_utn_edu_ar/Documents/Escritorio/Facultad/io/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mat\Desktop\TP-IO-main\TP-IO-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1019D43-3347-4AC3-B7A2-FCF292AB6F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D134F1F4-6068-4ADF-B1AF-D51B40F8A8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="17640" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESULTADOS ENVIOS (X)" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -603,14 +606,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D97"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -624,7 +627,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -635,10 +638,10 @@
         <v>5</v>
       </c>
       <c r="D2" s="6">
-        <v>546191.91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>635555.0572688696</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
@@ -652,7 +655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -666,7 +669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
@@ -680,7 +683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>3</v>
       </c>
@@ -694,7 +697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
@@ -708,7 +711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>3</v>
       </c>
@@ -719,10 +722,10 @@
         <v>7</v>
       </c>
       <c r="D8" s="8">
-        <v>218476.764</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+        <v>321191.34093000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>3</v>
       </c>
@@ -733,10 +736,10 @@
         <v>8</v>
       </c>
       <c r="D9" s="11">
-        <v>145651.17600000001</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+        <v>210048.18024500011</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>3</v>
       </c>
@@ -747,10 +750,10 @@
         <v>5</v>
       </c>
       <c r="D10" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+        <v>167423.2950561305</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>3</v>
       </c>
@@ -761,10 +764,10 @@
         <v>6</v>
       </c>
       <c r="D11" s="8">
-        <v>303439.95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+        <v>446099.08462500002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>3</v>
       </c>
@@ -778,7 +781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>3</v>
       </c>
@@ -789,10 +792,10 @@
         <v>8</v>
       </c>
       <c r="D13" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+        <v>4079.3803749998915</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>11</v>
       </c>
@@ -803,10 +806,10 @@
         <v>5</v>
       </c>
       <c r="D14" s="6">
-        <v>281371.58999999997</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>564444.9427311304</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>11</v>
       </c>
@@ -820,7 +823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>11</v>
       </c>
@@ -834,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>11</v>
       </c>
@@ -848,7 +851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>11</v>
       </c>
@@ -862,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>11</v>
       </c>
@@ -876,7 +879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>11</v>
       </c>
@@ -887,10 +890,10 @@
         <v>7</v>
       </c>
       <c r="D20" s="8">
-        <v>112548.63599999998</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+        <v>186139.79306999996</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>11</v>
       </c>
@@ -901,10 +904,10 @@
         <v>8</v>
       </c>
       <c r="D21" s="11">
-        <v>75032.423999999985</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+        <v>124093.19537999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>11</v>
       </c>
@@ -918,7 +921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>11</v>
       </c>
@@ -929,10 +932,10 @@
         <v>6</v>
       </c>
       <c r="D23" s="8">
-        <v>156317.54999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+        <v>258527.49037499996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>11</v>
       </c>
@@ -946,7 +949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>11</v>
       </c>
@@ -960,7 +963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>12</v>
       </c>
@@ -971,10 +974,10 @@
         <v>5</v>
       </c>
       <c r="D26" s="6">
-        <v>39919.5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>12</v>
       </c>
@@ -988,7 +991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>12</v>
       </c>
@@ -1002,7 +1005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>12</v>
       </c>
@@ -1016,7 +1019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>12</v>
       </c>
@@ -1030,7 +1033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>12</v>
       </c>
@@ -1044,7 +1047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>12</v>
       </c>
@@ -1055,10 +1058,10 @@
         <v>7</v>
       </c>
       <c r="D32" s="8">
-        <v>15967.8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+        <v>22591.19970999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>12</v>
       </c>
@@ -1069,10 +1072,10 @@
         <v>8</v>
       </c>
       <c r="D33" s="11">
-        <v>10645.199999999999</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>12</v>
       </c>
@@ -1083,10 +1086,10 @@
         <v>5</v>
       </c>
       <c r="D34" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+        <v>59666.039869499997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>12</v>
       </c>
@@ -1097,10 +1100,10 @@
         <v>6</v>
       </c>
       <c r="D35" s="8">
-        <v>22177.5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+        <v>33147.799927499997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>12</v>
       </c>
@@ -1111,10 +1114,10 @@
         <v>7</v>
       </c>
       <c r="D36" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1275.2162378000066</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
         <v>12</v>
       </c>
@@ -1125,10 +1128,10 @@
         <v>8</v>
       </c>
       <c r="D37" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+        <v>15910.943965199998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>13</v>
       </c>
@@ -1139,10 +1142,10 @@
         <v>5</v>
       </c>
       <c r="D38" s="6">
-        <v>114608.30437959186</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>13</v>
       </c>
@@ -1156,7 +1159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>13</v>
       </c>
@@ -1170,7 +1173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>13</v>
       </c>
@@ -1184,7 +1187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>13</v>
       </c>
@@ -1198,7 +1201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>13</v>
       </c>
@@ -1209,10 +1212,10 @@
         <v>6</v>
       </c>
       <c r="D43" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+        <v>88325.370290000006</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>13</v>
       </c>
@@ -1226,7 +1229,7 @@
         <v>5450.0579999999991</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>13</v>
       </c>
@@ -1240,7 +1243,7 @@
         <v>3633.3719999999998</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>13</v>
       </c>
@@ -1254,7 +1257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>13</v>
       </c>
@@ -1265,10 +1268,10 @@
         <v>6</v>
       </c>
       <c r="D47" s="8">
-        <v>7569.5249999999996</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>13</v>
       </c>
@@ -1282,7 +1285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>13</v>
       </c>
@@ -1296,7 +1299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>14</v>
       </c>
@@ -1307,10 +1310,10 @@
         <v>5</v>
       </c>
       <c r="D50" s="6">
-        <v>96808.5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+        <v>96770.7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>14</v>
       </c>
@@ -1321,10 +1324,10 @@
         <v>6</v>
       </c>
       <c r="D51" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+        <v>53229.3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>14</v>
       </c>
@@ -1338,7 +1341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>14</v>
       </c>
@@ -1352,7 +1355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>14</v>
       </c>
@@ -1366,7 +1369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>14</v>
       </c>
@@ -1377,10 +1380,10 @@
         <v>6</v>
       </c>
       <c r="D55" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+        <v>532.19999999999709</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>14</v>
       </c>
@@ -1391,10 +1394,10 @@
         <v>7</v>
       </c>
       <c r="D56" s="8">
-        <v>38723.4</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+        <v>38708.28</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>14</v>
       </c>
@@ -1405,10 +1408,10 @@
         <v>8</v>
       </c>
       <c r="D57" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+        <v>25805.52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>14</v>
       </c>
@@ -1422,7 +1425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>14</v>
       </c>
@@ -1433,10 +1436,10 @@
         <v>6</v>
       </c>
       <c r="D59" s="8">
-        <v>53782.5</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>14</v>
       </c>
@@ -1450,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
         <v>14</v>
       </c>
@@ -1461,10 +1464,10 @@
         <v>8</v>
       </c>
       <c r="D61" s="11">
-        <v>25815.599999999999</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>15</v>
       </c>
@@ -1475,10 +1478,10 @@
         <v>5</v>
       </c>
       <c r="D62" s="6">
-        <v>17995.5</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+        <v>28687.5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>15</v>
       </c>
@@ -1489,10 +1492,10 @@
         <v>6</v>
       </c>
       <c r="D63" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+        <v>6232.643254747918</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>15</v>
       </c>
@@ -1506,7 +1509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>15</v>
       </c>
@@ -1520,7 +1523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>15</v>
       </c>
@@ -1534,7 +1537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>15</v>
       </c>
@@ -1545,10 +1548,10 @@
         <v>6</v>
       </c>
       <c r="D67" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+        <v>9704.856745252082</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>15</v>
       </c>
@@ -1559,10 +1562,10 @@
         <v>7</v>
       </c>
       <c r="D68" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+        <v>11475</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>15</v>
       </c>
@@ -1573,10 +1576,10 @@
         <v>8</v>
       </c>
       <c r="D69" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+        <v>7650</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>15</v>
       </c>
@@ -1590,7 +1593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>15</v>
       </c>
@@ -1601,10 +1604,10 @@
         <v>6</v>
       </c>
       <c r="D71" s="8">
-        <v>9997.5</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>15</v>
       </c>
@@ -1615,10 +1618,10 @@
         <v>7</v>
       </c>
       <c r="D72" s="8">
-        <v>7198.2</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="9" t="s">
         <v>15</v>
       </c>
@@ -1629,10 +1632,10 @@
         <v>8</v>
       </c>
       <c r="D73" s="11">
-        <v>4798.8</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>16</v>
       </c>
@@ -1643,10 +1646,10 @@
         <v>5</v>
       </c>
       <c r="D74" s="6">
-        <v>218609.55000000002</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+        <v>218588.42249999999</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
         <v>16</v>
       </c>
@@ -1660,7 +1663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
         <v>16</v>
       </c>
@@ -1674,7 +1677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
         <v>16</v>
       </c>
@@ -1688,7 +1691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="7" t="s">
         <v>16</v>
       </c>
@@ -1702,7 +1705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>16</v>
       </c>
@@ -1716,7 +1719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
         <v>16</v>
       </c>
@@ -1727,10 +1730,10 @@
         <v>7</v>
       </c>
       <c r="D80" s="8">
-        <v>87443.819999999992</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+        <v>87435.368999999992</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
         <v>16</v>
       </c>
@@ -1741,10 +1744,10 @@
         <v>8</v>
       </c>
       <c r="D81" s="11">
-        <v>58295.88</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+        <v>58290.245999999999</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="7" t="s">
         <v>16</v>
       </c>
@@ -1758,7 +1761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
         <v>16</v>
       </c>
@@ -1769,10 +1772,10 @@
         <v>6</v>
       </c>
       <c r="D83" s="8">
-        <v>121449.75</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+        <v>121438.0125</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="7" t="s">
         <v>16</v>
       </c>
@@ -1786,7 +1789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="9" t="s">
         <v>16</v>
       </c>
@@ -1800,7 +1803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
         <v>17</v>
       </c>
@@ -1814,7 +1817,7 @@
         <v>70333.24500000001</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>17</v>
       </c>
@@ -1828,7 +1831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="7" t="s">
         <v>17</v>
       </c>
@@ -1842,7 +1845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
         <v>17</v>
       </c>
@@ -1856,7 +1859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="7" t="s">
         <v>17</v>
       </c>
@@ -1870,7 +1873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
         <v>17</v>
       </c>
@@ -1884,7 +1887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="7" t="s">
         <v>17</v>
       </c>
@@ -1898,7 +1901,7 @@
         <v>28133.297999999999</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
         <v>17</v>
       </c>
@@ -1912,7 +1915,7 @@
         <v>18755.531999999999</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="7" t="s">
         <v>17</v>
       </c>
@@ -1926,7 +1929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
         <v>17</v>
       </c>
@@ -1940,7 +1943,7 @@
         <v>39074.025000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="7" t="s">
         <v>17</v>
       </c>
@@ -1954,7 +1957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="9" t="s">
         <v>17</v>
       </c>
@@ -1976,12 +1979,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05649807-5BCA-4CDC-892B-C264250D9331}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1992,7 +1995,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2000,10 +2003,10 @@
         <v>21</v>
       </c>
       <c r="C2" s="15">
-        <v>4480622.5343550006</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>5477721.2427874999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -2011,10 +2014,10 @@
         <v>22</v>
       </c>
       <c r="C3" s="15">
-        <v>2262609.3395699998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>3728424.5855385503</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -2022,7 +2025,7 @@
         <v>23</v>
       </c>
       <c r="C4" s="15">
-        <v>1490206.4079749999</v>
+        <v>2592961.3613771666</v>
       </c>
     </row>
   </sheetData>
@@ -2033,14 +2036,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85634DFB-2640-45DB-972B-03B088998E42}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2051,7 +2054,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2059,10 +2062,10 @@
         <v>21</v>
       </c>
       <c r="C2" s="15">
-        <v>89559.050968955693</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -2070,7 +2073,7 @@
         <v>22</v>
       </c>
       <c r="C3" s="15">
-        <v>153989.61968015059</v>
+        <v>258527.49037499994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>